<commit_message>
Quantity per board added in PCBWay BOM
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/eSpark-BOM-v2.0 Boards_PCBWay.xlsx
+++ b/Deliverables/BOM/eSpark-BOM-v2.0 Boards_PCBWay.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25408"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\Melih-SoundSensor\Deliverables\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Faizan\GitHub\Melih-SoundSensor\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE9EB3AE-8AFA-4F59-A2FA-2EE31933FE47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="14010"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="240">
   <si>
     <t>S. No.</t>
   </si>
@@ -742,12 +741,15 @@
   </si>
   <si>
     <t>C2972450</t>
+  </si>
+  <si>
+    <t>Quantity (Per Board)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.0000"/>
   </numFmts>
@@ -895,36 +897,12 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="21">
+  <borders count="25">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom style="medium">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom style="medium">
-        <color auto="1"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -1165,6 +1143,84 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
@@ -1174,7 +1230,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="87">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1182,16 +1238,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1206,56 +1262,62 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1263,163 +1325,169 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="9" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="5" borderId="9" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="15" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="11" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="5" borderId="11" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="17" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="20" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="18" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1697,36 +1765,38 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I66"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:J66"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="6.109375" style="2" customWidth="1"/>
-    <col min="2" max="2" width="14.44140625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="47.5546875" style="9" customWidth="1"/>
-    <col min="4" max="4" width="35.109375" style="10" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="28.44140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="6.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.140625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="14.42578125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="47.5703125" style="9" customWidth="1"/>
+    <col min="4" max="4" width="35.140625" style="10" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="28.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6.42578125" style="2" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="16" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="9" style="1"/>
+    <col min="10" max="10" width="22.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="16.2" thickBot="1">
-      <c r="A1" s="79" t="s">
+    <row r="1" spans="1:10" ht="16.5" thickBot="1">
+      <c r="A1" s="81" t="s">
         <v>116</v>
       </c>
-      <c r="B1" s="80"/>
-      <c r="C1" s="80"/>
-      <c r="D1" s="80"/>
-      <c r="E1" s="80"/>
-      <c r="F1" s="80"/>
-      <c r="G1" s="80"/>
-      <c r="H1" s="80"/>
-      <c r="I1" s="80"/>
-    </row>
-    <row r="2" spans="1:9" ht="16.2" thickBot="1">
+      <c r="B1" s="82"/>
+      <c r="C1" s="82"/>
+      <c r="D1" s="82"/>
+      <c r="E1" s="82"/>
+      <c r="F1" s="82"/>
+      <c r="G1" s="82"/>
+      <c r="H1" s="82"/>
+      <c r="I1" s="82"/>
+      <c r="J1" s="82"/>
+    </row>
+    <row r="2" spans="1:10" ht="16.5" thickBot="1">
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
@@ -1754,8 +1824,11 @@
       <c r="I2" s="49" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" ht="15" thickBot="1">
+      <c r="J2" s="3" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="15.75" thickBot="1">
       <c r="A3" s="6">
         <v>1</v>
       </c>
@@ -1783,8 +1856,11 @@
       <c r="I3" s="13">
         <v>100</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" ht="15" thickBot="1">
+      <c r="J3" s="83">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="15.75" thickBot="1">
       <c r="A4" s="6">
         <v>2</v>
       </c>
@@ -1810,8 +1886,11 @@
       <c r="I4" s="17">
         <v>40</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" ht="42" thickBot="1">
+      <c r="J4" s="84">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="39" thickBot="1">
       <c r="A5" s="6">
         <v>3</v>
       </c>
@@ -1837,8 +1916,11 @@
       <c r="I5" s="17">
         <v>400</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" ht="15" thickBot="1">
+      <c r="J5" s="84">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="15.75" thickBot="1">
       <c r="A6" s="6">
         <v>4</v>
       </c>
@@ -1864,8 +1946,11 @@
       <c r="I6" s="17">
         <v>200</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" ht="15" thickBot="1">
+      <c r="J6" s="84">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="15.75" thickBot="1">
       <c r="A7" s="6">
         <v>5</v>
       </c>
@@ -1891,8 +1976,11 @@
       <c r="I7" s="17">
         <v>100</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" ht="55.8" thickBot="1">
+      <c r="J7" s="84">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="51.75" thickBot="1">
       <c r="A8" s="6">
         <v>6</v>
       </c>
@@ -1918,8 +2006,11 @@
       <c r="I8" s="17">
         <v>600</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" ht="15" thickBot="1">
+      <c r="J8" s="84">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="15.75" thickBot="1">
       <c r="A9" s="6">
         <v>7</v>
       </c>
@@ -1945,8 +2036,11 @@
       <c r="I9" s="18">
         <v>30</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" ht="15" thickBot="1">
+      <c r="J9" s="84">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="15.75" thickBot="1">
       <c r="A10" s="6">
         <v>8</v>
       </c>
@@ -1972,8 +2066,11 @@
       <c r="I10" s="18">
         <v>200</v>
       </c>
-    </row>
-    <row r="11" spans="1:9" ht="28.2" thickBot="1">
+      <c r="J10" s="84">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="26.25" thickBot="1">
       <c r="A11" s="6">
         <v>9</v>
       </c>
@@ -1999,8 +2096,11 @@
       <c r="I11" s="18">
         <v>350</v>
       </c>
-    </row>
-    <row r="12" spans="1:9" ht="15" thickBot="1">
+      <c r="J11" s="84">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="15.75" thickBot="1">
       <c r="A12" s="6">
         <v>10</v>
       </c>
@@ -2026,8 +2126,11 @@
       <c r="I12" s="18">
         <v>50</v>
       </c>
-    </row>
-    <row r="13" spans="1:9" ht="15" thickBot="1">
+      <c r="J12" s="84">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="15.75" thickBot="1">
       <c r="A13" s="6">
         <v>11</v>
       </c>
@@ -2053,8 +2156,11 @@
       <c r="I13" s="18">
         <v>100</v>
       </c>
-    </row>
-    <row r="14" spans="1:9" ht="15" thickBot="1">
+      <c r="J13" s="84">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="15.75" thickBot="1">
       <c r="A14" s="6">
         <v>12</v>
       </c>
@@ -2080,8 +2186,11 @@
       <c r="I14" s="18">
         <v>100</v>
       </c>
-    </row>
-    <row r="15" spans="1:9" ht="15" thickBot="1">
+      <c r="J14" s="84">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="15.75" thickBot="1">
       <c r="A15" s="6">
         <v>13</v>
       </c>
@@ -2107,8 +2216,11 @@
       <c r="I15" s="18">
         <v>50</v>
       </c>
-    </row>
-    <row r="16" spans="1:9" ht="15" thickBot="1">
+      <c r="J15" s="84">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="15.75" thickBot="1">
       <c r="A16" s="6">
         <v>14</v>
       </c>
@@ -2134,8 +2246,11 @@
       <c r="I16" s="18">
         <v>50</v>
       </c>
-    </row>
-    <row r="17" spans="1:9" ht="15" thickBot="1">
+      <c r="J16" s="84">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="15.75" thickBot="1">
       <c r="A17" s="6">
         <v>15</v>
       </c>
@@ -2161,12 +2276,15 @@
       <c r="I17" s="24">
         <v>50</v>
       </c>
-    </row>
-    <row r="18" spans="1:9" ht="28.2" thickBot="1">
+      <c r="J17" s="85">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="26.25" thickBot="1">
       <c r="A18" s="6">
         <v>16</v>
       </c>
-      <c r="B18" s="81" t="s">
+      <c r="B18" s="79" t="s">
         <v>148</v>
       </c>
       <c r="C18" s="50" t="s">
@@ -2190,12 +2308,15 @@
       <c r="I18" s="11">
         <v>30</v>
       </c>
-    </row>
-    <row r="19" spans="1:9" ht="15" thickBot="1">
+      <c r="J18" s="86">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="15.75" thickBot="1">
       <c r="A19" s="6">
         <v>17</v>
       </c>
-      <c r="B19" s="82"/>
+      <c r="B19" s="80"/>
       <c r="C19" s="51" t="s">
         <v>178</v>
       </c>
@@ -2217,8 +2338,11 @@
       <c r="I19" s="24">
         <v>50</v>
       </c>
-    </row>
-    <row r="20" spans="1:9" ht="15" thickBot="1">
+      <c r="J19" s="85">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="15.75" thickBot="1">
       <c r="A20" s="6">
         <v>18</v>
       </c>
@@ -2246,8 +2370,11 @@
       <c r="I20" s="11">
         <v>50</v>
       </c>
-    </row>
-    <row r="21" spans="1:9" ht="15" thickBot="1">
+      <c r="J20" s="86">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="15.75" thickBot="1">
       <c r="A21" s="6">
         <v>19</v>
       </c>
@@ -2273,8 +2400,11 @@
       <c r="I21" s="18">
         <v>45</v>
       </c>
-    </row>
-    <row r="22" spans="1:9" ht="15" thickBot="1">
+      <c r="J21" s="84">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="15.75" thickBot="1">
       <c r="A22" s="6">
         <v>20</v>
       </c>
@@ -2300,8 +2430,11 @@
       <c r="I22" s="18">
         <v>50</v>
       </c>
-    </row>
-    <row r="23" spans="1:9" ht="15" thickBot="1">
+      <c r="J22" s="84">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="15.75" thickBot="1">
       <c r="A23" s="6">
         <v>21</v>
       </c>
@@ -2327,8 +2460,11 @@
       <c r="I23" s="24">
         <v>30</v>
       </c>
-    </row>
-    <row r="24" spans="1:9" ht="28.2" thickBot="1">
+      <c r="J23" s="85">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="26.25" thickBot="1">
       <c r="A24" s="6">
         <v>22</v>
       </c>
@@ -2356,8 +2492,11 @@
       <c r="I24" s="60">
         <v>162</v>
       </c>
-    </row>
-    <row r="25" spans="1:9" ht="28.2" thickBot="1">
+      <c r="J24" s="86">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="26.25" thickBot="1">
       <c r="A25" s="6">
         <v>23</v>
       </c>
@@ -2385,8 +2524,11 @@
       <c r="I25" s="32">
         <v>30</v>
       </c>
-    </row>
-    <row r="26" spans="1:9" ht="28.2" thickBot="1">
+      <c r="J25" s="85">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="26.25" thickBot="1">
       <c r="A26" s="6">
         <v>24</v>
       </c>
@@ -2414,8 +2556,11 @@
       <c r="I26" s="23">
         <v>22</v>
       </c>
-    </row>
-    <row r="27" spans="1:9" ht="28.2" thickBot="1">
+      <c r="J26" s="86">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="26.25" thickBot="1">
       <c r="A27" s="6">
         <v>25</v>
       </c>
@@ -2441,8 +2586,11 @@
       <c r="I27" s="17">
         <v>45</v>
       </c>
-    </row>
-    <row r="28" spans="1:9" ht="28.2" thickBot="1">
+      <c r="J27" s="84">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" ht="26.25" thickBot="1">
       <c r="A28" s="6">
         <v>26</v>
       </c>
@@ -2468,8 +2616,11 @@
       <c r="I28" s="26">
         <v>25</v>
       </c>
-    </row>
-    <row r="29" spans="1:9" ht="15" thickBot="1">
+      <c r="J28" s="85">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="15.75" thickBot="1">
       <c r="A29" s="6">
         <v>27</v>
       </c>
@@ -2497,8 +2648,11 @@
       <c r="I29" s="53">
         <v>100</v>
       </c>
-    </row>
-    <row r="30" spans="1:9" ht="15" thickBot="1">
+      <c r="J29" s="86">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="15.75" thickBot="1">
       <c r="A30" s="6">
         <v>28</v>
       </c>
@@ -2524,8 +2678,11 @@
       <c r="I30" s="37">
         <v>100</v>
       </c>
-    </row>
-    <row r="31" spans="1:9" ht="15" thickBot="1">
+      <c r="J30" s="84">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="15.75" thickBot="1">
       <c r="A31" s="6">
         <v>29</v>
       </c>
@@ -2551,8 +2708,11 @@
       <c r="I31" s="37">
         <v>100</v>
       </c>
-    </row>
-    <row r="32" spans="1:9" ht="15" thickBot="1">
+      <c r="J31" s="84">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" ht="15.75" thickBot="1">
       <c r="A32" s="6">
         <v>30</v>
       </c>
@@ -2578,8 +2738,11 @@
       <c r="I32" s="37">
         <v>100</v>
       </c>
-    </row>
-    <row r="33" spans="1:9" ht="15" thickBot="1">
+      <c r="J32" s="84">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" ht="15.75" thickBot="1">
       <c r="A33" s="6">
         <v>31</v>
       </c>
@@ -2605,8 +2768,11 @@
       <c r="I33" s="55">
         <v>100</v>
       </c>
-    </row>
-    <row r="34" spans="1:9" ht="15" thickBot="1">
+      <c r="J33" s="85">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="15.75" thickBot="1">
       <c r="A34" s="6">
         <v>32</v>
       </c>
@@ -2634,8 +2800,11 @@
       <c r="I34" s="13">
         <v>42</v>
       </c>
-    </row>
-    <row r="35" spans="1:9" ht="28.2" thickBot="1">
+      <c r="J34" s="86">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" ht="26.25" thickBot="1">
       <c r="A35" s="6">
         <v>33</v>
       </c>
@@ -2661,8 +2830,11 @@
       <c r="I35" s="16">
         <v>21</v>
       </c>
-    </row>
-    <row r="36" spans="1:9" ht="15" thickBot="1">
+      <c r="J35" s="84">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" ht="15.75" thickBot="1">
       <c r="A36" s="6">
         <v>34</v>
       </c>
@@ -2688,8 +2860,11 @@
       <c r="I36" s="18">
         <v>21</v>
       </c>
-    </row>
-    <row r="37" spans="1:9" ht="15" thickBot="1">
+      <c r="J36" s="84">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" ht="15.75" thickBot="1">
       <c r="A37" s="6">
         <v>35</v>
       </c>
@@ -2715,8 +2890,11 @@
       <c r="I37" s="18">
         <v>41</v>
       </c>
-    </row>
-    <row r="38" spans="1:9" ht="15" thickBot="1">
+      <c r="J37" s="84">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" ht="15.75" thickBot="1">
       <c r="A38" s="6">
         <v>36</v>
       </c>
@@ -2742,8 +2920,11 @@
       <c r="I38" s="18">
         <v>21</v>
       </c>
-    </row>
-    <row r="39" spans="1:9" ht="15" thickBot="1">
+      <c r="J38" s="84">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" ht="15.75" thickBot="1">
       <c r="A39" s="6">
         <v>37</v>
       </c>
@@ -2769,8 +2950,11 @@
       <c r="I39" s="18">
         <v>21</v>
       </c>
-    </row>
-    <row r="40" spans="1:9" ht="15" thickBot="1">
+      <c r="J39" s="84">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" ht="15.75" thickBot="1">
       <c r="A40" s="6">
         <v>38</v>
       </c>
@@ -2796,8 +2980,11 @@
       <c r="I40" s="18">
         <v>22</v>
       </c>
-    </row>
-    <row r="41" spans="1:9" ht="15" thickBot="1">
+      <c r="J40" s="84">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" ht="15.75" thickBot="1">
       <c r="A41" s="6">
         <v>39</v>
       </c>
@@ -2823,8 +3010,11 @@
       <c r="I41" s="20">
         <v>30</v>
       </c>
-    </row>
-    <row r="42" spans="1:9" ht="28.2" thickBot="1">
+      <c r="J41" s="84">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" ht="26.25" thickBot="1">
       <c r="A42" s="6">
         <v>40</v>
       </c>
@@ -2850,8 +3040,11 @@
       <c r="I42" s="24">
         <v>30</v>
       </c>
-    </row>
-    <row r="43" spans="1:9" ht="15" thickBot="1">
+      <c r="J42" s="85">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" ht="15.75" thickBot="1">
       <c r="A43" s="6">
         <v>41</v>
       </c>
@@ -2879,8 +3072,11 @@
       <c r="I43" s="27">
         <v>50</v>
       </c>
-    </row>
-    <row r="44" spans="1:9" ht="28.2" thickBot="1">
+      <c r="J43" s="86">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" ht="26.25" thickBot="1">
       <c r="A44" s="6">
         <v>42</v>
       </c>
@@ -2906,8 +3102,11 @@
       <c r="I44" s="17">
         <v>30</v>
       </c>
-    </row>
-    <row r="45" spans="1:9" ht="15" thickBot="1">
+      <c r="J44" s="84">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" ht="15.75" thickBot="1">
       <c r="A45" s="6">
         <v>43</v>
       </c>
@@ -2933,8 +3132,11 @@
       <c r="I45" s="17">
         <v>50</v>
       </c>
-    </row>
-    <row r="46" spans="1:9" ht="15" thickBot="1">
+      <c r="J45" s="84">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" ht="15.75" thickBot="1">
       <c r="A46" s="6">
         <v>44</v>
       </c>
@@ -2960,8 +3162,11 @@
       <c r="I46" s="17">
         <v>25</v>
       </c>
-    </row>
-    <row r="47" spans="1:9" ht="15" thickBot="1">
+      <c r="J46" s="84">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" ht="15.75" thickBot="1">
       <c r="A47" s="6">
         <v>45</v>
       </c>
@@ -2987,8 +3192,11 @@
       <c r="I47" s="32">
         <v>40</v>
       </c>
-    </row>
-    <row r="48" spans="1:9" ht="111" thickBot="1">
+      <c r="J47" s="84">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" ht="102.75" thickBot="1">
       <c r="A48" s="6">
         <v>46</v>
       </c>
@@ -3012,8 +3220,11 @@
       <c r="I48" s="44" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="49" spans="1:9" ht="28.2" thickBot="1">
+      <c r="J48" s="85">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" ht="26.25" thickBot="1">
       <c r="A49" s="6">
         <v>47</v>
       </c>
@@ -3041,8 +3252,11 @@
       <c r="I49" s="63" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="50" spans="1:9" ht="15" thickBot="1">
+      <c r="J49" s="86">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" ht="15.75" thickBot="1">
       <c r="A50" s="72">
         <v>48</v>
       </c>
@@ -3068,63 +3282,66 @@
       <c r="I50" s="65" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="51" spans="1:9">
+      <c r="J50" s="85">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10">
       <c r="A51" s="1"/>
       <c r="C51" s="2"/>
       <c r="D51" s="2"/>
       <c r="I51" s="7"/>
     </row>
-    <row r="52" spans="1:9">
+    <row r="52" spans="1:10">
       <c r="A52" s="1"/>
       <c r="C52" s="2"/>
       <c r="D52" s="2"/>
       <c r="I52" s="7"/>
     </row>
-    <row r="53" spans="1:9">
+    <row r="53" spans="1:10">
       <c r="A53" s="1"/>
       <c r="C53" s="2"/>
       <c r="D53" s="2"/>
     </row>
-    <row r="54" spans="1:9">
+    <row r="54" spans="1:10">
       <c r="A54" s="1"/>
       <c r="C54" s="2"/>
       <c r="D54" s="2"/>
     </row>
-    <row r="55" spans="1:9">
+    <row r="55" spans="1:10">
       <c r="A55" s="1"/>
       <c r="C55" s="2"/>
       <c r="D55" s="2"/>
     </row>
-    <row r="56" spans="1:9">
+    <row r="56" spans="1:10">
       <c r="A56" s="1"/>
       <c r="C56" s="2"/>
       <c r="D56" s="2"/>
     </row>
-    <row r="57" spans="1:9">
+    <row r="57" spans="1:10">
       <c r="A57" s="1"/>
       <c r="C57" s="2"/>
       <c r="D57" s="2"/>
     </row>
-    <row r="58" spans="1:9">
+    <row r="58" spans="1:10">
       <c r="A58" s="1"/>
     </row>
-    <row r="59" spans="1:9" ht="15.75" customHeight="1">
+    <row r="59" spans="1:10" ht="15.75" customHeight="1">
       <c r="A59" s="1"/>
     </row>
-    <row r="60" spans="1:9">
+    <row r="60" spans="1:10">
       <c r="A60" s="1"/>
     </row>
-    <row r="61" spans="1:9">
+    <row r="61" spans="1:10">
       <c r="A61" s="1"/>
     </row>
-    <row r="62" spans="1:9">
+    <row r="62" spans="1:10">
       <c r="A62" s="1"/>
     </row>
-    <row r="63" spans="1:9">
+    <row r="63" spans="1:10">
       <c r="A63" s="1"/>
     </row>
-    <row r="64" spans="1:9">
+    <row r="64" spans="1:10">
       <c r="A64" s="1"/>
     </row>
     <row r="65" spans="7:7">
@@ -3138,16 +3355,16 @@
     <mergeCell ref="B49:B50"/>
     <mergeCell ref="B3:B17"/>
     <mergeCell ref="B20:B23"/>
-    <mergeCell ref="A1:I1"/>
     <mergeCell ref="B29:B33"/>
     <mergeCell ref="B34:B42"/>
     <mergeCell ref="B43:B48"/>
     <mergeCell ref="B26:B28"/>
     <mergeCell ref="B18:B19"/>
+    <mergeCell ref="A1:J1"/>
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="I48">
-    <cfRule type="dataBar" priority="54">
+    <cfRule type="dataBar" priority="59">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>

</xml_diff>